<commit_message>
fix: Tool-Bugs aus User-Review
Rebalancing_Tool:
- Spalte J (Fehlbetrag) für Aktien: IF(P=0; 0; I-F) → bei eingefrorener Sparrate (FLAG/D1) auch kein Nachkauf-Signal mehr. MSFT + APH Fehlbetrag fällt jetzt konsistent auf 0€.

Satelliten_Monitor:
- Spalte Q (Score-Datum): Datetime-Objekte zu Text-Strings '17.04.2026' korrigiert (Zelle hatte Text-Format → #### / falsche Darstellung).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Rebalancing_Tool_v3.4.xlsx
+++ b/03_Tools/Rebalancing_Tool_v3.4.xlsx
@@ -1381,7 +1381,7 @@
         <v/>
       </c>
       <c r="J10" s="17">
-        <f>I10-F10</f>
+        <f>IF(P10=0,0,I10-F10)</f>
         <v/>
       </c>
       <c r="K10" s="18">
@@ -1450,7 +1450,7 @@
         <v/>
       </c>
       <c r="J11" s="23">
-        <f>I11-F11</f>
+        <f>IF(P11=0,0,I11-F11)</f>
         <v/>
       </c>
       <c r="K11" s="24">
@@ -1519,7 +1519,7 @@
         <v/>
       </c>
       <c r="J12" s="17">
-        <f>I12-F12</f>
+        <f>IF(P12=0,0,I12-F12)</f>
         <v/>
       </c>
       <c r="K12" s="18">
@@ -1588,7 +1588,7 @@
         <v/>
       </c>
       <c r="J13" s="23">
-        <f>I13-F13</f>
+        <f>IF(P13=0,0,I13-F13)</f>
         <v/>
       </c>
       <c r="K13" s="24">
@@ -1657,7 +1657,7 @@
         <v/>
       </c>
       <c r="J14" s="17">
-        <f>I14-F14</f>
+        <f>IF(P14=0,0,I14-F14)</f>
         <v/>
       </c>
       <c r="K14" s="18">
@@ -1726,7 +1726,7 @@
         <v/>
       </c>
       <c r="J15" s="23">
-        <f>I15-F15</f>
+        <f>IF(P15=0,0,I15-F15)</f>
         <v/>
       </c>
       <c r="K15" s="24">
@@ -1795,7 +1795,7 @@
         <v/>
       </c>
       <c r="J16" s="17">
-        <f>I16-F16</f>
+        <f>IF(P16=0,0,I16-F16)</f>
         <v/>
       </c>
       <c r="K16" s="18">
@@ -1864,7 +1864,7 @@
         <v/>
       </c>
       <c r="J17" s="23">
-        <f>I17-F17</f>
+        <f>IF(P17=0,0,I17-F17)</f>
         <v/>
       </c>
       <c r="K17" s="24">
@@ -1933,7 +1933,7 @@
         <v/>
       </c>
       <c r="J18" s="17">
-        <f>I18-F18</f>
+        <f>IF(P18=0,0,I18-F18)</f>
         <v/>
       </c>
       <c r="K18" s="18">
@@ -2002,7 +2002,7 @@
         <v/>
       </c>
       <c r="J19" s="23">
-        <f>I19-F19</f>
+        <f>IF(P19=0,0,I19-F19)</f>
         <v/>
       </c>
       <c r="K19" s="24">
@@ -2071,7 +2071,7 @@
         <v/>
       </c>
       <c r="J20" s="17">
-        <f>I20-F20</f>
+        <f>IF(P20=0,0,I20-F20)</f>
         <v/>
       </c>
       <c r="K20" s="18">

</xml_diff>

<commit_message>
Vault + Tools + Skills Sync: v3.7 Post-ASML-Update Abschluss
Vault (9 Dateien):
- 7 Satellite-Entities (APH/ASML/AVGO/MSFT/RMS/SU/TMO): v3.7-Scores, Frontmatter, Historie
- sources/dynastie-depot-skill.md: D3-Rate-Fix (D4/D3=1.0, D2=0.5, FLAG=0.0), Nenner 8.5
- synthesis/Wissenschaftliche-Fundierung-DEFCON.md: v3.5-Zeitstand-Banner (B-konform)
- sources/Jadhav-Mirza-2025.md, concepts/defcon/Analyse-Pipeline.md, log.md

Tools:
- Rebalancing_Tool_v3.4.xlsx: APH Score 66->68 (N10/O10)
- Satelliten_Monitor_v2.0.xlsx: ASML 66->68, APH-Text 61->63, QuickScreen-Legende 17.04.
- 03_Tools/portfolio_risk.py NEU (aus _extern/risk-metrics-calculation extrahiert)
- 03_Tools/Output/PORTFOLIO-RISK-2026-04-17.md

Skills:
- dynastie-depot/config.yaml: ASML 66->68, scoring_notiz v3.7, MSFT flag_grund
- dynastie-depot/SKILL.md + PIPELINE.md + Beispiele.md: v3.7-Header, ASML-Anker
- _extern/earnings-calendar geloescht

CLAUDE.md: Applied Learning Updates
</commit_message>
<xml_diff>
--- a/03_Tools/Rebalancing_Tool_v3.4.xlsx
+++ b/03_Tools/Rebalancing_Tool_v3.4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tobia\OneDrive\Desktop\Claude Stuff\03_Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6202B1A-E672-4754-8C99-DF3C7E3D451E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8340C460-79F7-476E-B969-07D07C16950D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio &amp; Rebalancing" sheetId="1" r:id="rId1"/>
@@ -149,10 +149,10 @@
     <t>Aktie</t>
   </si>
   <si>
-    <t>DEFCON 3 (66)</t>
-  </si>
-  <si>
-    <t>🟡 DEFCON 3 (66) | China Rev 14.7% Risk-Map</t>
+    <t>DEFCON 3 (68)</t>
+  </si>
+  <si>
+    <t>🟡 DEFCON 3 (68) | China Rev 14.7% Risk-Map</t>
   </si>
   <si>
     <t>Broadcom</t>
@@ -663,7 +663,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -829,13 +829,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -844,6 +842,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1323,44 +1330,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
     </row>
     <row r="2" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="70">
+      <c r="A2" s="68">
         <v>46129</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
+      <c r="N2" s="67"/>
+      <c r="O2" s="67"/>
+      <c r="P2" s="67"/>
     </row>
     <row r="3" spans="1:16" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -2929,8 +2936,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.85546875" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -3150,11 +3157,11 @@
       <c r="A25" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="B25" s="61">
+      <c r="B25" s="70">
         <f>B4*B6</f>
         <v>285</v>
       </c>
-      <c r="C25" s="62" t="s">
+      <c r="C25" s="61" t="s">
         <v>96</v>
       </c>
     </row>
@@ -3162,68 +3169,68 @@
       <c r="A26" s="60" t="s">
         <v>126</v>
       </c>
-      <c r="B26" s="63">
+      <c r="B26" s="62">
         <f>COUNTIFS('Portfolio &amp; Rebalancing'!C5:C20,"Aktie",'Portfolio &amp; Rebalancing'!N5:N20,"DEFCON 4*",'Portfolio &amp; Rebalancing'!O5:O20,"&lt;&gt;🔴*")+COUNTIFS('Portfolio &amp; Rebalancing'!C5:C20,"Aktie",'Portfolio &amp; Rebalancing'!N5:N20,"DEFCON 3*",'Portfolio &amp; Rebalancing'!O5:O20,"&lt;&gt;🔴*")</f>
         <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="64" t="s">
+      <c r="A27" s="63" t="s">
         <v>127</v>
       </c>
-      <c r="B27" s="65">
+      <c r="B27" s="71">
         <v>0.5</v>
       </c>
-      <c r="C27" s="64" t="s">
+      <c r="C27" s="69" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="66" t="s">
+      <c r="A28" s="64" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="64" t="s">
+      <c r="A29" s="63" t="s">
         <v>129</v>
       </c>
-      <c r="B29" s="67" t="s">
+      <c r="B29" s="65" t="s">
         <v>130</v>
       </c>
-      <c r="C29" s="64" t="s">
+      <c r="C29" s="63" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="64" t="s">
+      <c r="A30" s="63" t="s">
         <v>132</v>
       </c>
-      <c r="B30" s="67" t="s">
+      <c r="B30" s="65" t="s">
         <v>133</v>
       </c>
-      <c r="C30" s="64" t="s">
+      <c r="C30" s="63" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="64" t="s">
+      <c r="A31" s="63" t="s">
         <v>135</v>
       </c>
-      <c r="B31" s="67" t="s">
+      <c r="B31" s="65" t="s">
         <v>136</v>
       </c>
-      <c r="C31" s="64" t="s">
+      <c r="C31" s="63" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="64" t="s">
+      <c r="A32" s="63" t="s">
         <v>138</v>
       </c>
-      <c r="B32" s="67" t="s">
+      <c r="B32" s="65" t="s">
         <v>136</v>
       </c>
-      <c r="C32" s="64" t="s">
+      <c r="C32" s="63" t="s">
         <v>139</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(rebalancing): Positionswerte ING + Scalable aktualisiert (Stand 18.04.2026)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Rebalancing_Tool_v3.4.xlsx
+++ b/03_Tools/Rebalancing_Tool_v3.4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tobia\OneDrive\Desktop\Claude Stuff\03_Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8340C460-79F7-476E-B969-07D07C16950D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE8D108-ECB4-417F-B3F5-91C9530772C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio &amp; Rebalancing" sheetId="1" r:id="rId1"/>
@@ -836,21 +836,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1330,44 +1330,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
     </row>
     <row r="2" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="68">
+      <c r="A2" s="71">
         <v>46129</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
-      <c r="O2" s="67"/>
-      <c r="P2" s="67"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="70"/>
+      <c r="M2" s="70"/>
+      <c r="N2" s="70"/>
+      <c r="O2" s="70"/>
+      <c r="P2" s="70"/>
     </row>
     <row r="3" spans="1:16" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -1437,26 +1437,26 @@
         <v>0</v>
       </c>
       <c r="F5" s="5">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="G5" s="6">
         <f t="shared" ref="G5:G20" si="0">IF(F$25=0,0,F5/F$25)</f>
-        <v>4.4812648657344099E-2</v>
+        <v>4.304963260382038E-2</v>
       </c>
       <c r="H5" s="6">
         <v>0.05</v>
       </c>
       <c r="I5" s="5">
         <f t="shared" ref="I5:I20" si="1">H5*F$25</f>
-        <v>565.68850000000009</v>
+        <v>593.50100000000009</v>
       </c>
       <c r="J5" s="5">
         <f>I5-F5</f>
-        <v>58.68850000000009</v>
+        <v>82.50100000000009</v>
       </c>
       <c r="K5" s="6">
         <f t="shared" ref="K5:K20" si="2">G5-H5</f>
-        <v>-5.1873513426559034E-3</v>
+        <v>-6.9503673961796228E-3</v>
       </c>
       <c r="L5" s="3" t="str">
         <f>IF(C5="Aktie",IF(K5&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K5&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K5&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K5&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1490,26 +1490,26 @@
         <v>0.7</v>
       </c>
       <c r="F6" s="11">
-        <v>2792.3</v>
+        <v>2960.39</v>
       </c>
       <c r="G6" s="12">
         <f t="shared" si="0"/>
-        <v>0.24680544151065473</v>
+        <v>0.24940059073194482</v>
       </c>
       <c r="H6" s="12">
         <v>0.3</v>
       </c>
       <c r="I6" s="11">
         <f t="shared" si="1"/>
-        <v>3394.1309999999999</v>
+        <v>3561.0059999999999</v>
       </c>
       <c r="J6" s="11">
         <f>I6-F6</f>
-        <v>601.83099999999968</v>
+        <v>600.61599999999999</v>
       </c>
       <c r="K6" s="12">
         <f t="shared" si="2"/>
-        <v>-5.3194558489345262E-2</v>
+        <v>-5.0599409268055173E-2</v>
       </c>
       <c r="L6" s="9" t="str">
         <f>IF(C6="Aktie",IF(K6&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K6&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K6&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K6&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1543,26 +1543,26 @@
         <v>0</v>
       </c>
       <c r="F7" s="11">
-        <v>913.01</v>
+        <v>1002.95</v>
       </c>
       <c r="G7" s="12">
         <f t="shared" si="0"/>
-        <v>8.0699006608760823E-2</v>
+        <v>8.4494381643838851E-2</v>
       </c>
       <c r="H7" s="12">
         <v>0.1</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="1"/>
-        <v>1131.3770000000002</v>
+        <v>1187.0020000000002</v>
       </c>
       <c r="J7" s="11">
         <f>I7-F7</f>
-        <v>218.36700000000019</v>
+        <v>184.05200000000013</v>
       </c>
       <c r="K7" s="12">
         <f t="shared" si="2"/>
-        <v>-1.9300993391239182E-2</v>
+        <v>-1.5505618356161155E-2</v>
       </c>
       <c r="L7" s="9" t="str">
         <f>IF(C7="Aktie",IF(K7&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K7&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K7&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K7&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1596,26 +1596,26 @@
         <v>0</v>
       </c>
       <c r="F8" s="11">
-        <v>917.46</v>
+        <v>955.68</v>
       </c>
       <c r="G8" s="12">
         <f t="shared" si="0"/>
-        <v>8.1092332617686239E-2</v>
+        <v>8.0512080013344534E-2</v>
       </c>
       <c r="H8" s="12">
         <v>0.15</v>
       </c>
       <c r="I8" s="11">
         <f t="shared" si="1"/>
-        <v>1697.0654999999999</v>
+        <v>1780.5029999999999</v>
       </c>
       <c r="J8" s="11">
         <f>I8-F8</f>
-        <v>779.60549999999989</v>
+        <v>824.82299999999998</v>
       </c>
       <c r="K8" s="12">
         <f t="shared" si="2"/>
-        <v>-6.8907667382313756E-2</v>
+        <v>-6.9487919986655461E-2</v>
       </c>
       <c r="L8" s="9" t="str">
         <f>IF(C8="Aktie",IF(K8&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K8&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K8&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K8&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1653,26 +1653,26 @@
       </c>
       <c r="G9" s="12">
         <f t="shared" si="0"/>
-        <v>8.8476255041422966E-2</v>
+        <v>8.4330102223922107E-2</v>
       </c>
       <c r="H9" s="12">
         <v>0.1</v>
       </c>
       <c r="I9" s="11">
         <f t="shared" si="1"/>
-        <v>1131.3770000000002</v>
+        <v>1187.0020000000002</v>
       </c>
       <c r="J9" s="11">
         <f>I9-F9</f>
-        <v>130.37700000000018</v>
+        <v>186.00200000000018</v>
       </c>
       <c r="K9" s="12">
         <f t="shared" si="2"/>
-        <v>-1.152374495857704E-2</v>
+        <v>-1.5669897776077898E-2</v>
       </c>
       <c r="L9" s="9" t="str">
         <f>IF(C9="Aktie",IF(K9&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K9&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K9&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K9&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
-        <v>⚖️ Halten</v>
+        <v>📈 Aufstocken</v>
       </c>
       <c r="M9" s="13" t="str">
         <f>IF(C9="Aktie",IF(G9&gt;'Parameter &amp; Regeln'!B$10,"🚨 ÜBER CAP","✅ OK"),"")</f>
@@ -1702,26 +1702,26 @@
         <v>0</v>
       </c>
       <c r="F10" s="17">
-        <v>364</v>
+        <v>388</v>
       </c>
       <c r="G10" s="18">
         <f t="shared" si="0"/>
-        <v>3.2173183651426532E-2</v>
+        <v>3.2687392270611168E-2</v>
       </c>
       <c r="H10" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I10" s="17">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J10" s="17">
         <f t="shared" ref="J10:J20" si="3">IF(P10=0,0,I10-F10)</f>
-        <v>-55.134078999999986</v>
+        <v>-63.94845399999997</v>
       </c>
       <c r="K10" s="18">
         <f t="shared" si="2"/>
-        <v>4.8731836514265305E-3</v>
+        <v>5.3873922706111667E-3</v>
       </c>
       <c r="L10" s="15" t="str">
         <f>IF(C10="Aktie",IF(K10&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K10&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K10&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K10&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1759,26 +1759,26 @@
         <v>1</v>
       </c>
       <c r="F11" s="23">
-        <v>356</v>
+        <v>453</v>
       </c>
       <c r="G11" s="24">
         <f t="shared" si="0"/>
-        <v>3.1466080714032542E-2</v>
+        <v>3.8163372934502213E-2</v>
       </c>
       <c r="H11" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I11" s="23">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J11" s="23">
         <f t="shared" si="3"/>
-        <v>-47.134078999999986</v>
+        <v>-128.94845399999997</v>
       </c>
       <c r="K11" s="24">
         <f t="shared" si="2"/>
-        <v>4.1660807140325405E-3</v>
+        <v>1.0863372934502211E-2</v>
       </c>
       <c r="L11" s="21" t="str">
         <f>IF(C11="Aktie",IF(K11&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K11&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K11&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K11&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1816,18 +1816,18 @@
         <v>1</v>
       </c>
       <c r="F12" s="17">
-        <v>301</v>
+        <v>333</v>
       </c>
       <c r="G12" s="18">
         <f t="shared" si="0"/>
-        <v>2.6604748019448864E-2</v>
+        <v>2.8053870170395668E-2</v>
       </c>
       <c r="H12" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I12" s="17">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J12" s="17">
         <f t="shared" si="3"/>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="K12" s="18">
         <f t="shared" si="2"/>
-        <v>-6.9525198055113771E-4</v>
+        <v>7.5387017039566656E-4</v>
       </c>
       <c r="L12" s="15" t="str">
         <f>IF(C12="Aktie",IF(K12&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K12&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K12&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K12&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1873,26 +1873,26 @@
         <v>1</v>
       </c>
       <c r="F13" s="23">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="G13" s="24">
         <f t="shared" si="0"/>
-        <v>3.0935753510987051E-2</v>
+        <v>2.9149066303173876E-2</v>
       </c>
       <c r="H13" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I13" s="23">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J13" s="23">
         <f t="shared" si="3"/>
-        <v>-41.134078999999986</v>
+        <v>-21.94845399999997</v>
       </c>
       <c r="K13" s="24">
         <f t="shared" si="2"/>
-        <v>3.6357535109870498E-3</v>
+        <v>1.8490663031738748E-3</v>
       </c>
       <c r="L13" s="21" t="str">
         <f>IF(C13="Aktie",IF(K13&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K13&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K13&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K13&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1930,26 +1930,26 @@
         <v>0</v>
       </c>
       <c r="F14" s="17">
-        <v>377</v>
+        <v>396</v>
       </c>
       <c r="G14" s="18">
         <f t="shared" si="0"/>
-        <v>3.3322225924691772E-2</v>
+        <v>3.3361359121551602E-2</v>
       </c>
       <c r="H14" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I14" s="17">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J14" s="17">
         <f t="shared" si="3"/>
-        <v>-68.134078999999986</v>
+        <v>-71.94845399999997</v>
       </c>
       <c r="K14" s="18">
         <f t="shared" si="2"/>
-        <v>6.0222259246917702E-3</v>
+        <v>6.0613591215516009E-3</v>
       </c>
       <c r="L14" s="15" t="str">
         <f>IF(C14="Aktie",IF(K14&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K14&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K14&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K14&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1987,26 +1987,26 @@
         <v>1</v>
       </c>
       <c r="F15" s="23">
-        <v>323</v>
+        <v>302</v>
       </c>
       <c r="G15" s="24">
         <f t="shared" si="0"/>
-        <v>2.8549281097282338E-2</v>
+        <v>2.5442248623001477E-2</v>
       </c>
       <c r="H15" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I15" s="23">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J15" s="23">
         <f t="shared" si="3"/>
-        <v>-14.134078999999986</v>
+        <v>22.05154600000003</v>
       </c>
       <c r="K15" s="24">
         <f t="shared" si="2"/>
-        <v>1.2492810972823364E-3</v>
+        <v>-1.8577513769985239E-3</v>
       </c>
       <c r="L15" s="21" t="str">
         <f>IF(C15="Aktie",IF(K15&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K15&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K15&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K15&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2044,26 +2044,26 @@
         <v>0</v>
       </c>
       <c r="F16" s="17">
-        <v>336</v>
+        <v>390</v>
       </c>
       <c r="G16" s="18">
         <f t="shared" si="0"/>
-        <v>2.969832337054757E-2</v>
+        <v>3.2855883983346275E-2</v>
       </c>
       <c r="H16" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I16" s="17">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J16" s="17">
         <f t="shared" si="3"/>
-        <v>-27.134078999999986</v>
+        <v>-65.94845399999997</v>
       </c>
       <c r="K16" s="18">
         <f t="shared" si="2"/>
-        <v>2.3983233705475691E-3</v>
+        <v>5.5558839833462735E-3</v>
       </c>
       <c r="L16" s="15" t="str">
         <f>IF(C16="Aktie",IF(K16&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K16&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K16&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K16&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2101,26 +2101,26 @@
         <v>1</v>
       </c>
       <c r="F17" s="23">
-        <v>403</v>
+        <v>392</v>
       </c>
       <c r="G17" s="24">
         <f t="shared" si="0"/>
-        <v>3.5620310471222237E-2</v>
+        <v>3.3024375696081389E-2</v>
       </c>
       <c r="H17" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I17" s="23">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J17" s="23">
         <f t="shared" si="3"/>
-        <v>-94.134078999999986</v>
+        <v>-67.94845399999997</v>
       </c>
       <c r="K17" s="24">
         <f t="shared" si="2"/>
-        <v>8.3203104712222357E-3</v>
+        <v>5.7243756960813873E-3</v>
       </c>
       <c r="L17" s="21" t="str">
         <f>IF(C17="Aktie",IF(K17&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K17&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K17&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K17&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2158,26 +2158,26 @@
         <v>1</v>
       </c>
       <c r="F18" s="17">
-        <v>416</v>
+        <v>427</v>
       </c>
       <c r="G18" s="18">
         <f t="shared" si="0"/>
-        <v>3.676935274448747E-2</v>
+        <v>3.5972980668945796E-2</v>
       </c>
       <c r="H18" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I18" s="17">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J18" s="17">
         <f t="shared" si="3"/>
-        <v>-107.13407899999999</v>
+        <v>-102.94845399999997</v>
       </c>
       <c r="K18" s="18">
         <f t="shared" si="2"/>
-        <v>9.4693527444874685E-3</v>
+        <v>8.6729806689457949E-3</v>
       </c>
       <c r="L18" s="15" t="str">
         <f>IF(C18="Aktie",IF(K18&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K18&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K18&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K18&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2215,26 +2215,26 @@
         <v>1</v>
       </c>
       <c r="F19" s="23">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="G19" s="24">
         <f t="shared" si="0"/>
-        <v>2.280406973095617E-2</v>
+        <v>2.274638121923973E-2</v>
       </c>
       <c r="H19" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I19" s="23">
         <f t="shared" si="1"/>
-        <v>308.86592100000001</v>
+        <v>324.05154600000003</v>
       </c>
       <c r="J19" s="23">
         <f t="shared" si="3"/>
-        <v>50.865921000000014</v>
+        <v>54.05154600000003</v>
       </c>
       <c r="K19" s="24">
         <f t="shared" si="2"/>
-        <v>-4.495930269043831E-3</v>
+        <v>-4.5536187807602713E-3</v>
       </c>
       <c r="L19" s="21" t="str">
         <f>IF(C19="Aktie",IF(K19&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K19&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K19&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K19&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2272,18 +2272,18 @@
         <v>1</v>
       </c>
       <c r="F20" s="17">
-        <v>249</v>
+        <v>292</v>
       </c>
       <c r="G20" s="18">
         <f t="shared" si="0"/>
-        <v>2.2008578926387933E-2</v>
+        <v>2.4599790059325929E-2</v>
       </c>
       <c r="H20" s="18">
         <v>2.7E-2</v>
       </c>
       <c r="I20" s="17">
         <f t="shared" si="1"/>
-        <v>305.47179</v>
+        <v>320.49054000000001</v>
       </c>
       <c r="J20" s="17">
         <f t="shared" si="3"/>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="K20" s="18">
         <f t="shared" si="2"/>
-        <v>-4.9914210736120672E-3</v>
+        <v>-2.4002099406740703E-3</v>
       </c>
       <c r="L20" s="15" t="str">
         <f>IF(C20="Aktie",IF(K20&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K20&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K20&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K20&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2322,11 +2322,11 @@
       <c r="E21" s="27"/>
       <c r="F21" s="28">
         <f>SUM(F5:F20)</f>
-        <v>9863.77</v>
+        <v>10420.02</v>
       </c>
       <c r="G21" s="29">
         <f>SUM(G5:G20)</f>
-        <v>0.87183759259733951</v>
+        <v>0.87784350826704582</v>
       </c>
       <c r="H21" s="29">
         <f>SUM(H5:H20)</f>
@@ -2334,15 +2334,15 @@
       </c>
       <c r="I21" s="28">
         <f>SUM(I5:I20)</f>
-        <v>11313.770000000004</v>
+        <v>11870.020000000006</v>
       </c>
       <c r="J21" s="28">
         <f>ROUND(SUM(J5:J20),2)</f>
-        <v>1385.66</v>
+        <v>1430.46</v>
       </c>
       <c r="K21" s="29">
         <f>SUMPRODUCT((C5:C20="Aktie")*ABS(K5:K20))/COUNTIF(C5:C20,"Aktie")</f>
-        <v>4.5742831643531398E-3</v>
+        <v>4.8799892042764408E-3</v>
       </c>
       <c r="L21" s="26" t="s">
         <v>72</v>
@@ -2367,7 +2367,7 @@
     <row r="22" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K22" s="32">
         <f>SUMPRODUCT((C5:C20&lt;&gt;"Aktie")*ABS(K5:K20))/COUNTIF(C5:C20,"&lt;&gt;Aktie")</f>
-        <v>3.1622863112826229E-2</v>
+        <v>3.1642642556625869E-2</v>
       </c>
       <c r="L22" s="33" t="s">
         <v>73</v>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="F25" s="41">
         <f>F21 + F24</f>
-        <v>11313.77</v>
+        <v>11870.02</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="F26" s="42">
         <f>F24 - MIN(F23, SUMIFS(J5:J20, D5:D20, "Scalable", J5:J20, "&gt;0"))</f>
-        <v>1210.0685789999998</v>
+        <v>1105.3939079999996</v>
       </c>
     </row>
   </sheetData>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="C4" s="47">
         <f>'Portfolio &amp; Rebalancing'!F5</f>
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="D4" s="48">
         <f>'Portfolio &amp; Rebalancing'!E5</f>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="C5" s="47">
         <f>'Portfolio &amp; Rebalancing'!F6</f>
-        <v>2792.3</v>
+        <v>2960.39</v>
       </c>
       <c r="D5" s="48">
         <f>'Portfolio &amp; Rebalancing'!E6</f>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="E5" s="47">
         <f t="shared" si="0"/>
-        <v>1954.61</v>
+        <v>2072.2729999999997</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="C6" s="47">
         <f>'Portfolio &amp; Rebalancing'!F7</f>
-        <v>913.01</v>
+        <v>1002.95</v>
       </c>
       <c r="D6" s="48">
         <f>'Portfolio &amp; Rebalancing'!E7</f>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C7" s="47">
         <f>'Portfolio &amp; Rebalancing'!F8</f>
-        <v>917.46</v>
+        <v>955.68</v>
       </c>
       <c r="D7" s="48">
         <f>'Portfolio &amp; Rebalancing'!E8</f>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C9" s="47">
         <f>'Portfolio &amp; Rebalancing'!F10</f>
-        <v>364</v>
+        <v>388</v>
       </c>
       <c r="D9" s="48">
         <f>'Portfolio &amp; Rebalancing'!E10</f>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="C10" s="47">
         <f>'Portfolio &amp; Rebalancing'!F11</f>
-        <v>356</v>
+        <v>453</v>
       </c>
       <c r="D10" s="48">
         <f>'Portfolio &amp; Rebalancing'!E11</f>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="E10" s="47">
         <f t="shared" si="0"/>
-        <v>356</v>
+        <v>453</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="C11" s="47">
         <f>'Portfolio &amp; Rebalancing'!F12</f>
-        <v>301</v>
+        <v>333</v>
       </c>
       <c r="D11" s="48">
         <f>'Portfolio &amp; Rebalancing'!E12</f>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="E11" s="47">
         <f t="shared" si="0"/>
-        <v>301</v>
+        <v>333</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C12" s="47">
         <f>'Portfolio &amp; Rebalancing'!F13</f>
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="D12" s="48">
         <f>'Portfolio &amp; Rebalancing'!E13</f>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="E12" s="47">
         <f t="shared" si="0"/>
-        <v>350</v>
+        <v>346</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C13" s="47">
         <f>'Portfolio &amp; Rebalancing'!F14</f>
-        <v>377</v>
+        <v>396</v>
       </c>
       <c r="D13" s="48">
         <f>'Portfolio &amp; Rebalancing'!E14</f>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="C14" s="47">
         <f>'Portfolio &amp; Rebalancing'!F15</f>
-        <v>323</v>
+        <v>302</v>
       </c>
       <c r="D14" s="48">
         <f>'Portfolio &amp; Rebalancing'!E15</f>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="E14" s="47">
         <f t="shared" si="0"/>
-        <v>323</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="C15" s="47">
         <f>'Portfolio &amp; Rebalancing'!F16</f>
-        <v>336</v>
+        <v>390</v>
       </c>
       <c r="D15" s="48">
         <f>'Portfolio &amp; Rebalancing'!E16</f>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="C16" s="47">
         <f>'Portfolio &amp; Rebalancing'!F17</f>
-        <v>403</v>
+        <v>392</v>
       </c>
       <c r="D16" s="48">
         <f>'Portfolio &amp; Rebalancing'!E17</f>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="E16" s="47">
         <f t="shared" si="0"/>
-        <v>403</v>
+        <v>392</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="C17" s="47">
         <f>'Portfolio &amp; Rebalancing'!F18</f>
-        <v>416</v>
+        <v>427</v>
       </c>
       <c r="D17" s="48">
         <f>'Portfolio &amp; Rebalancing'!E18</f>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="E17" s="47">
         <f t="shared" si="0"/>
-        <v>416</v>
+        <v>427</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C18" s="47">
         <f>'Portfolio &amp; Rebalancing'!F19</f>
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="D18" s="48">
         <f>'Portfolio &amp; Rebalancing'!E19</f>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="E18" s="47">
         <f t="shared" si="0"/>
-        <v>258</v>
+        <v>270</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="C19" s="47">
         <f>'Portfolio &amp; Rebalancing'!F20</f>
-        <v>249</v>
+        <v>292</v>
       </c>
       <c r="D19" s="48">
         <f>'Portfolio &amp; Rebalancing'!E20</f>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="E19" s="47">
         <f t="shared" si="0"/>
-        <v>249</v>
+        <v>292</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="C20" s="50">
         <f>'Portfolio &amp; Rebalancing'!F21</f>
-        <v>9863.77</v>
+        <v>10420.02</v>
       </c>
       <c r="E20" s="50">
         <f>SUM(E4:E19)</f>
-        <v>5281.28</v>
+        <v>5557.9429999999993</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="B22" s="51">
         <f>IF('Portfolio &amp; Rebalancing'!F25=0,0,E20/'Portfolio &amp; Rebalancing'!F25)</f>
-        <v>0.46680107515001629</v>
+        <v>0.46823366767705521</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="B23" s="51">
         <f>SUMPRODUCT('Portfolio &amp; Rebalancing'!$E$5:$E$20,'Portfolio &amp; Rebalancing'!$I$5:$I$20)/SUM('Portfolio &amp; Rebalancing'!$I$5:$I$20)</f>
-        <v>0.49509999999999971</v>
+        <v>0.4950999999999996</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -3157,7 +3157,7 @@
       <c r="A25" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="B25" s="70">
+      <c r="B25" s="67">
         <f>B4*B6</f>
         <v>285</v>
       </c>
@@ -3178,10 +3178,10 @@
       <c r="A27" s="63" t="s">
         <v>127</v>
       </c>
-      <c r="B27" s="71">
+      <c r="B27" s="68">
         <v>0.5</v>
       </c>
-      <c r="C27" s="69" t="s">
+      <c r="C27" s="66" t="s">
         <v>98</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(tools): Emoji-CF-Regeln auf LEFT(1) — APH rote Färbung wiederhergestellt
**Ursache:** Modernes Excel (365/2021+) ist bei LEFT() **codepoint-basiert**
— mein Fix vorher nutzte LEFT(O,2)="🔴" und LEFT(O,2)="🚩" in der Annahme
UTF-16-Code-Units. Das matcht aber nicht, weil LEFT(2) "🔴 " (emoji + Leerz.)
zurückgibt statt des nackten "🔴".

**Fix:** Alle Emoji-CF-Regeln auf `LEFT(...,1)="<emoji>"` vereinheitlicht.

Betroffen:
- Rebal O5:O20: 🔴 und 🚩 waren "tot" → APH (O20 "🔴 FLAG...") ungefärbt
- Monitor N7:N17: gleiche Normalisierung zur Konsistenz

V/TMO (🟠) funktionierten bereits korrekt weil ich dort schon LEFT(1) hatte.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Rebalancing_Tool_v3.4.xlsx
+++ b/03_Tools/Rebalancing_Tool_v3.4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tobia\OneDrive\Desktop\Claude Stuff\03_Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB7FC57-15D8-4DED-B222-8C170299C3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CB7F22-2BA9-4B90-B318-C26D0D2EB6C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2492,20 +2492,20 @@
     <cfRule type="expression" dxfId="8" priority="19" stopIfTrue="1">
       <formula>O5="✅ Clean"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="20" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="19" stopIfTrue="1">
       <formula>LEFT(O5,1)="🟢"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="21" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="19" stopIfTrue="1">
       <formula>LEFT(O5,1)="🟡"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="22" stopIfTrue="1">
-      <formula>LEFT(O5,2)="🚩"</formula>
+    <cfRule type="expression" dxfId="5" priority="20" stopIfTrue="1">
+      <formula>LEFT(O5,1)="🚩"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="23" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="21" stopIfTrue="1">
       <formula>LEFT(O5,1)="🟠"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="24" stopIfTrue="1">
-      <formula>LEFT(O5,2)="🔴"</formula>
+    <cfRule type="expression" dxfId="3" priority="22" stopIfTrue="1">
+      <formula>LEFT(O5,1)="🔴"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5:P20">

</xml_diff>

<commit_message>
chore(tool): Rebalancing_Tool_v3.4.xlsx — aktuelle Positions-Werte eingetragen (scoring-neutral)
User-Eingabe aktueller Positions-/Kurswerte ins Rebalancing-Tool.
Operativer Daten-Refresh, KEIN Score/FLAG/Sparraten-Event → eigenständiger
Tool-Commit (CLAUDE.md §18), kein 8-File-Sync. xlsx-smoke-test §18.7 PASS.
DEFCON v3.7 + 11 Scores + Sparraten 285EUR unverändert.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Rebalancing_Tool_v3.4.xlsx
+++ b/03_Tools/Rebalancing_Tool_v3.4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tobia\OneDrive\Desktop\Claude Stuff\03_Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3F8EE2-41B4-48A0-9DDE-896F929C3E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E59FF7EA-2373-4173-8164-449484EA10F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1475,26 +1475,26 @@
         <v>0</v>
       </c>
       <c r="F5" s="5">
-        <v>594</v>
+        <v>582</v>
       </c>
       <c r="G5" s="6">
         <f t="shared" ref="G5:G20" si="0">IF(F$25=0,0,F5/F$25)</f>
-        <v>4.2834489407838426E-2</v>
+        <v>4.221839532376867E-2</v>
       </c>
       <c r="H5" s="6">
         <v>0.05</v>
       </c>
       <c r="I5" s="5">
         <f t="shared" ref="I5:I20" si="1">H5*F$25</f>
-        <v>693.36649999999997</v>
+        <v>689.27300000000002</v>
       </c>
       <c r="J5" s="5">
         <f>I5-F5</f>
-        <v>99.366499999999974</v>
+        <v>107.27300000000002</v>
       </c>
       <c r="K5" s="6">
         <f t="shared" ref="K5:K20" si="2">G5-H5</f>
-        <v>-7.1655105921615767E-3</v>
+        <v>-7.7816046762313323E-3</v>
       </c>
       <c r="L5" s="3" t="str">
         <f>IF(C5="Aktie",IF(K5&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K5&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K5&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K5&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1528,26 +1528,26 @@
         <v>0.7</v>
       </c>
       <c r="F6" s="11">
-        <v>3632.72</v>
+        <v>3675.72</v>
       </c>
       <c r="G6" s="12">
         <f t="shared" si="0"/>
-        <v>0.26196246862229428</v>
+        <v>0.26663745714687792</v>
       </c>
       <c r="H6" s="12">
         <v>0.3</v>
       </c>
       <c r="I6" s="11">
         <f t="shared" si="1"/>
-        <v>4160.1989999999996</v>
+        <v>4135.6379999999999</v>
       </c>
       <c r="J6" s="11">
         <f>I6-F6</f>
-        <v>527.47899999999981</v>
+        <v>459.91800000000012</v>
       </c>
       <c r="K6" s="12">
         <f t="shared" si="2"/>
-        <v>-3.8037531377705713E-2</v>
+        <v>-3.3362542853122068E-2</v>
       </c>
       <c r="L6" s="9" t="str">
         <f>IF(C6="Aktie",IF(K6&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K6&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K6&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K6&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1581,26 +1581,26 @@
         <v>0</v>
       </c>
       <c r="F7" s="11">
-        <v>1246.4100000000001</v>
+        <v>1228.3</v>
       </c>
       <c r="G7" s="12">
         <f t="shared" si="0"/>
-        <v>8.9881036940780978E-2</v>
+        <v>8.9101125388634114E-2</v>
       </c>
       <c r="H7" s="12">
         <v>0.1</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="1"/>
-        <v>1386.7329999999999</v>
+        <v>1378.546</v>
       </c>
       <c r="J7" s="11">
         <f>I7-F7</f>
-        <v>140.32299999999987</v>
+        <v>150.24600000000009</v>
       </c>
       <c r="K7" s="12">
         <f t="shared" si="2"/>
-        <v>-1.0118963059219027E-2</v>
+        <v>-1.0898874611365891E-2</v>
       </c>
       <c r="L7" s="9" t="str">
         <f>IF(C7="Aktie",IF(K7&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K7&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K7&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K7&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1634,26 +1634,26 @@
         <v>0</v>
       </c>
       <c r="F8" s="11">
-        <v>1800.2</v>
+        <v>1769.44</v>
       </c>
       <c r="G8" s="12">
         <f t="shared" si="0"/>
-        <v>0.12981590544106186</v>
+        <v>0.12835552821596088</v>
       </c>
       <c r="H8" s="12">
         <v>0.15</v>
       </c>
       <c r="I8" s="11">
         <f t="shared" si="1"/>
-        <v>2080.0994999999998</v>
+        <v>2067.819</v>
       </c>
       <c r="J8" s="11">
         <f>I8-F8</f>
-        <v>279.89949999999976</v>
+        <v>298.37899999999991</v>
       </c>
       <c r="K8" s="12">
         <f t="shared" si="2"/>
-        <v>-2.0184094558938132E-2</v>
+        <v>-2.164447178403911E-2</v>
       </c>
       <c r="L8" s="9" t="str">
         <f>IF(C8="Aktie",IF(K8&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K8&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K8&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K8&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1687,26 +1687,26 @@
         <v>0.67</v>
       </c>
       <c r="F9" s="11">
-        <v>1194</v>
+        <v>1187</v>
       </c>
       <c r="G9" s="12">
         <f t="shared" si="0"/>
-        <v>8.6101650425857046E-2</v>
+        <v>8.6105215205005858E-2</v>
       </c>
       <c r="H9" s="12">
         <v>0.1</v>
       </c>
       <c r="I9" s="11">
         <f t="shared" si="1"/>
-        <v>1386.7329999999999</v>
+        <v>1378.546</v>
       </c>
       <c r="J9" s="11">
         <f>I9-F9</f>
-        <v>192.73299999999995</v>
+        <v>191.54600000000005</v>
       </c>
       <c r="K9" s="12">
         <f t="shared" si="2"/>
-        <v>-1.389834957414296E-2</v>
+        <v>-1.3894784794994147E-2</v>
       </c>
       <c r="L9" s="9" t="str">
         <f>IF(C9="Aktie",IF(K9&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K9&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K9&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K9&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1740,26 +1740,26 @@
         <v>0</v>
       </c>
       <c r="F10" s="17">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="G10" s="18">
         <f t="shared" si="0"/>
-        <v>3.1657139478183619E-2</v>
+        <v>3.2135307780806734E-2</v>
       </c>
       <c r="H10" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I10" s="17">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J10" s="17">
         <f t="shared" ref="J10:J20" si="3">IF(P10=0,0,I10-F10)</f>
-        <v>-60.421891000000016</v>
+        <v>-66.656942000000015</v>
       </c>
       <c r="K10" s="18">
         <f t="shared" si="2"/>
-        <v>4.3571394781836172E-3</v>
+        <v>4.8353077808067323E-3</v>
       </c>
       <c r="L10" s="15" t="str">
         <f>IF(C10="Aktie",IF(K10&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K10&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K10&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K10&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1797,18 +1797,18 @@
         <v>1</v>
       </c>
       <c r="F11" s="23">
-        <v>506</v>
+        <v>516</v>
       </c>
       <c r="G11" s="24">
         <f t="shared" si="0"/>
-        <v>3.6488639125195697E-2</v>
+        <v>3.7430742245815524E-2</v>
       </c>
       <c r="H11" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I11" s="23">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J11" s="23">
         <f t="shared" si="3"/>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="K11" s="24">
         <f t="shared" si="2"/>
-        <v>9.188639125195696E-3</v>
+        <v>1.0130742245815522E-2</v>
       </c>
       <c r="L11" s="21" t="str">
         <f>IF(C11="Aktie",IF(K11&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K11&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K11&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K11&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1854,18 +1854,18 @@
         <v>1</v>
       </c>
       <c r="F12" s="17">
-        <v>376</v>
+        <v>387</v>
       </c>
       <c r="G12" s="18">
         <f t="shared" si="0"/>
-        <v>2.7114087571291665E-2</v>
+        <v>2.8073056684361639E-2</v>
       </c>
       <c r="H12" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I12" s="17">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J12" s="17">
         <f t="shared" si="3"/>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="K12" s="18">
         <f t="shared" si="2"/>
-        <v>-1.8591242870833607E-4</v>
+        <v>7.7305668436163794E-4</v>
       </c>
       <c r="L12" s="15" t="str">
         <f>IF(C12="Aktie",IF(K12&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K12&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K12&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K12&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1911,26 +1911,26 @@
         <v>1</v>
       </c>
       <c r="F13" s="23">
-        <v>384</v>
+        <v>404</v>
       </c>
       <c r="G13" s="24">
         <f t="shared" si="0"/>
-        <v>2.7690983051531913E-2</v>
+        <v>2.9306240052925332E-2</v>
       </c>
       <c r="H13" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I13" s="23">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J13" s="23">
         <f t="shared" si="3"/>
-        <v>-5.4218910000000164</v>
+        <v>-27.656942000000015</v>
       </c>
       <c r="K13" s="24">
         <f t="shared" si="2"/>
-        <v>3.9098305153191168E-4</v>
+        <v>2.0062400529253302E-3</v>
       </c>
       <c r="L13" s="21" t="str">
         <f>IF(C13="Aktie",IF(K13&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K13&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K13&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K13&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1968,26 +1968,26 @@
         <v>0</v>
       </c>
       <c r="F14" s="17">
-        <v>420</v>
+        <v>394</v>
       </c>
       <c r="G14" s="18">
         <f t="shared" si="0"/>
-        <v>3.028701271261303E-2</v>
+        <v>2.8580838071417279E-2</v>
       </c>
       <c r="H14" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I14" s="17">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J14" s="17">
         <f t="shared" si="3"/>
-        <v>-41.421891000000016</v>
+        <v>-17.656942000000015</v>
       </c>
       <c r="K14" s="18">
         <f t="shared" si="2"/>
-        <v>2.9870127126130283E-3</v>
+        <v>1.2808380714172778E-3</v>
       </c>
       <c r="L14" s="15" t="str">
         <f>IF(C14="Aktie",IF(K14&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K14&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K14&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K14&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2025,26 +2025,26 @@
         <v>1</v>
       </c>
       <c r="F15" s="23">
-        <v>342</v>
+        <v>322</v>
       </c>
       <c r="G15" s="24">
         <f t="shared" si="0"/>
-        <v>2.466228178027061E-2</v>
+        <v>2.3357943804559297E-2</v>
       </c>
       <c r="H15" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I15" s="23">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J15" s="23">
         <f t="shared" si="3"/>
-        <v>36.578108999999984</v>
+        <v>54.343057999999985</v>
       </c>
       <c r="K15" s="24">
         <f t="shared" si="2"/>
-        <v>-2.6377182197293916E-3</v>
+        <v>-3.9420561954407046E-3</v>
       </c>
       <c r="L15" s="21" t="str">
         <f>IF(C15="Aktie",IF(K15&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K15&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K15&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K15&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2082,26 +2082,26 @@
         <v>0</v>
       </c>
       <c r="F16" s="17">
-        <v>434</v>
+        <v>407</v>
       </c>
       <c r="G16" s="18">
         <f t="shared" si="0"/>
-        <v>3.1296579803033464E-2</v>
+        <v>2.9523860647377748E-2</v>
       </c>
       <c r="H16" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I16" s="17">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J16" s="17">
         <f t="shared" si="3"/>
-        <v>-55.421891000000016</v>
+        <v>-30.656942000000015</v>
       </c>
       <c r="K16" s="18">
         <f t="shared" si="2"/>
-        <v>3.9965798030334627E-3</v>
+        <v>2.2238606473777463E-3</v>
       </c>
       <c r="L16" s="15" t="str">
         <f>IF(C16="Aktie",IF(K16&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K16&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K16&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K16&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2139,26 +2139,26 @@
         <v>1</v>
       </c>
       <c r="F17" s="23">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="G17" s="24">
         <f t="shared" si="0"/>
-        <v>3.0575460452733155E-2</v>
+        <v>3.1917687186354321E-2</v>
       </c>
       <c r="H17" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I17" s="23">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J17" s="23">
         <f t="shared" si="3"/>
-        <v>-45.421891000000016</v>
+        <v>-63.656942000000015</v>
       </c>
       <c r="K17" s="24">
         <f t="shared" si="2"/>
-        <v>3.2754604527331539E-3</v>
+        <v>4.6176871863543197E-3</v>
       </c>
       <c r="L17" s="21" t="str">
         <f>IF(C17="Aktie",IF(K17&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K17&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K17&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K17&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2196,26 +2196,26 @@
         <v>1</v>
       </c>
       <c r="F18" s="17">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="G18" s="18">
         <f t="shared" si="0"/>
-        <v>3.4036833334174642E-2</v>
+        <v>3.4674214716084922E-2</v>
       </c>
       <c r="H18" s="18">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I18" s="17">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J18" s="17">
         <f t="shared" si="3"/>
-        <v>-93.421891000000016</v>
+        <v>-101.65694200000002</v>
       </c>
       <c r="K18" s="18">
         <f t="shared" si="2"/>
-        <v>6.7368333341746404E-3</v>
+        <v>7.374214716084921E-3</v>
       </c>
       <c r="L18" s="15" t="str">
         <f>IF(C18="Aktie",IF(K18&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K18&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K18&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K18&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2253,26 +2253,26 @@
         <v>1</v>
       </c>
       <c r="F19" s="23">
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="G19" s="24">
         <f t="shared" si="0"/>
-        <v>2.3436378884760082E-2</v>
+        <v>2.2124760435995608E-2</v>
       </c>
       <c r="H19" s="24">
         <v>2.7300000000000001E-2</v>
       </c>
       <c r="I19" s="23">
         <f t="shared" si="1"/>
-        <v>378.57810899999998</v>
+        <v>376.34305799999998</v>
       </c>
       <c r="J19" s="23">
         <f t="shared" si="3"/>
-        <v>53.578108999999984</v>
+        <v>71.343057999999985</v>
       </c>
       <c r="K19" s="24">
         <f t="shared" si="2"/>
-        <v>-3.8636211152399194E-3</v>
+        <v>-5.1752395640043934E-3</v>
       </c>
       <c r="L19" s="21" t="str">
         <f>IF(C19="Aktie",IF(K19&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K19&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K19&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K19&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2310,18 +2310,18 @@
         <v>1</v>
       </c>
       <c r="F20" s="17">
-        <v>328</v>
+        <v>297</v>
       </c>
       <c r="G20" s="18">
         <f t="shared" si="0"/>
-        <v>2.3652714689850175E-2</v>
+        <v>2.1544438850789167E-2</v>
       </c>
       <c r="H20" s="18">
         <v>2.7E-2</v>
       </c>
       <c r="I20" s="17">
         <f t="shared" si="1"/>
-        <v>374.41790999999995</v>
+        <v>372.20741999999996</v>
       </c>
       <c r="J20" s="17">
         <f t="shared" si="3"/>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="K20" s="18">
         <f t="shared" si="2"/>
-        <v>-3.3472853101498244E-3</v>
+        <v>-5.4555611492108323E-3</v>
       </c>
       <c r="L20" s="15" t="str">
         <f>IF(C20="Aktie",IF(K20&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K20&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K20&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K20&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2360,11 +2360,11 @@
       <c r="E21" s="27"/>
       <c r="F21" s="28">
         <f>SUM(F5:F20)</f>
-        <v>12917.329999999998</v>
+        <v>12835.46</v>
       </c>
       <c r="G21" s="29">
         <f>SUM(G5:G20)</f>
-        <v>0.93149366172147074</v>
+        <v>0.93108681175673524</v>
       </c>
       <c r="H21" s="29">
         <f>SUM(H5:H20)</f>
@@ -2372,15 +2372,15 @@
       </c>
       <c r="I21" s="28">
         <f>SUM(I5:I20)</f>
-        <v>13867.33</v>
+        <v>13785.460000000005</v>
       </c>
       <c r="J21" s="28">
         <f>ROUND(SUM(J5:J20),2)</f>
-        <v>1028.43</v>
+        <v>1025.1099999999999</v>
       </c>
       <c r="K21" s="29">
         <f>SUMPRODUCT((C5:C20="Aktie")*ABS(K5:K20))/COUNTIF(C5:C20,"Aktie")</f>
-        <v>3.7242895482993625E-3</v>
+        <v>4.3468003903454015E-3</v>
       </c>
       <c r="L21" s="26" t="s">
         <v>74</v>
@@ -2405,7 +2405,7 @@
     <row r="22" spans="1:16" ht="16.5" customHeight="1">
       <c r="K22" s="32">
         <f>SUMPRODUCT((C5:C20&lt;&gt;"Aktie")*ABS(K5:K20))/COUNTIF(C5:C20,"&lt;&gt;Aktie")</f>
-        <v>1.7880889832433484E-2</v>
+        <v>1.7516455743950509E-2</v>
       </c>
       <c r="L22" s="33" t="s">
         <v>75</v>
@@ -2429,7 +2429,7 @@
         <v>79</v>
       </c>
       <c r="F23" s="38">
-        <v>1291.77</v>
+        <v>1297.78</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="16.5" customHeight="1">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="F25" s="41">
         <f>F21 + F24</f>
-        <v>13867.329999999998</v>
+        <v>13785.46</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="16.5" customHeight="1">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F26" s="42">
         <f>F24 - MIN(F23, SUMIFS(J5:J20, D5:D20, "Scalable", J5:J20, "&gt;0"))</f>
-        <v>567.74428200000011</v>
+        <v>525.49488399999996</v>
       </c>
     </row>
   </sheetData>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="C4" s="47">
         <f>'Portfolio &amp; Rebalancing'!F5</f>
-        <v>594</v>
+        <v>582</v>
       </c>
       <c r="D4" s="48">
         <f>'Portfolio &amp; Rebalancing'!E5</f>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C5" s="47">
         <f>'Portfolio &amp; Rebalancing'!F6</f>
-        <v>3632.72</v>
+        <v>3675.72</v>
       </c>
       <c r="D5" s="48">
         <f>'Portfolio &amp; Rebalancing'!E6</f>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="E5" s="47">
         <f t="shared" si="0"/>
-        <v>2542.9039999999995</v>
+        <v>2573.0039999999999</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C6" s="47">
         <f>'Portfolio &amp; Rebalancing'!F7</f>
-        <v>1246.4100000000001</v>
+        <v>1228.3</v>
       </c>
       <c r="D6" s="48">
         <f>'Portfolio &amp; Rebalancing'!E7</f>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C7" s="47">
         <f>'Portfolio &amp; Rebalancing'!F8</f>
-        <v>1800.2</v>
+        <v>1769.44</v>
       </c>
       <c r="D7" s="48">
         <f>'Portfolio &amp; Rebalancing'!E8</f>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="C8" s="47">
         <f>'Portfolio &amp; Rebalancing'!F9</f>
-        <v>1194</v>
+        <v>1187</v>
       </c>
       <c r="D8" s="48">
         <f>'Portfolio &amp; Rebalancing'!E9</f>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="E8" s="47">
         <f t="shared" si="0"/>
-        <v>799.98</v>
+        <v>795.29000000000008</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="C9" s="47">
         <f>'Portfolio &amp; Rebalancing'!F10</f>
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="D9" s="48">
         <f>'Portfolio &amp; Rebalancing'!E10</f>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C10" s="47">
         <f>'Portfolio &amp; Rebalancing'!F11</f>
-        <v>506</v>
+        <v>516</v>
       </c>
       <c r="D10" s="48">
         <f>'Portfolio &amp; Rebalancing'!E11</f>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="E10" s="47">
         <f t="shared" si="0"/>
-        <v>506</v>
+        <v>516</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C11" s="47">
         <f>'Portfolio &amp; Rebalancing'!F12</f>
-        <v>376</v>
+        <v>387</v>
       </c>
       <c r="D11" s="48">
         <f>'Portfolio &amp; Rebalancing'!E12</f>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="E11" s="47">
         <f t="shared" si="0"/>
-        <v>376</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="C12" s="47">
         <f>'Portfolio &amp; Rebalancing'!F13</f>
-        <v>384</v>
+        <v>404</v>
       </c>
       <c r="D12" s="48">
         <f>'Portfolio &amp; Rebalancing'!E13</f>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="E12" s="47">
         <f t="shared" si="0"/>
-        <v>384</v>
+        <v>404</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="C13" s="47">
         <f>'Portfolio &amp; Rebalancing'!F14</f>
-        <v>420</v>
+        <v>394</v>
       </c>
       <c r="D13" s="48">
         <f>'Portfolio &amp; Rebalancing'!E14</f>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="C14" s="47">
         <f>'Portfolio &amp; Rebalancing'!F15</f>
-        <v>342</v>
+        <v>322</v>
       </c>
       <c r="D14" s="48">
         <f>'Portfolio &amp; Rebalancing'!E15</f>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="E14" s="47">
         <f t="shared" si="0"/>
-        <v>342</v>
+        <v>322</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="C15" s="47">
         <f>'Portfolio &amp; Rebalancing'!F16</f>
-        <v>434</v>
+        <v>407</v>
       </c>
       <c r="D15" s="48">
         <f>'Portfolio &amp; Rebalancing'!E16</f>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C16" s="47">
         <f>'Portfolio &amp; Rebalancing'!F17</f>
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="D16" s="48">
         <f>'Portfolio &amp; Rebalancing'!E17</f>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="E16" s="47">
         <f t="shared" si="0"/>
-        <v>424</v>
+        <v>440</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="C17" s="47">
         <f>'Portfolio &amp; Rebalancing'!F18</f>
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="D17" s="48">
         <f>'Portfolio &amp; Rebalancing'!E18</f>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="E17" s="47">
         <f t="shared" si="0"/>
-        <v>472</v>
+        <v>478</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="C18" s="47">
         <f>'Portfolio &amp; Rebalancing'!F19</f>
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="D18" s="48">
         <f>'Portfolio &amp; Rebalancing'!E19</f>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="E18" s="47">
         <f t="shared" si="0"/>
-        <v>325</v>
+        <v>305</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="C19" s="47">
         <f>'Portfolio &amp; Rebalancing'!F20</f>
-        <v>328</v>
+        <v>297</v>
       </c>
       <c r="D19" s="48">
         <f>'Portfolio &amp; Rebalancing'!E20</f>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="E19" s="47">
         <f t="shared" si="0"/>
-        <v>328</v>
+        <v>297</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2917,11 +2917,11 @@
       </c>
       <c r="C20" s="50">
         <f>'Portfolio &amp; Rebalancing'!F21</f>
-        <v>12917.329999999998</v>
+        <v>12835.46</v>
       </c>
       <c r="E20" s="50">
         <f>SUM(E4:E19)</f>
-        <v>6499.884</v>
+        <v>6517.2939999999999</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="B22" s="51">
         <f>IF('Portfolio &amp; Rebalancing'!F25=0,0,E20/'Portfolio &amp; Rebalancing'!F25)</f>
-        <v>0.46871921271073819</v>
+        <v>0.47276579816705427</v>
       </c>
     </row>
     <row r="23" spans="1:5">

</xml_diff>

<commit_message>
chore(03_Tools): Rebalancing_Tool Beträge-Update (User-Edit)
Sparbeträge-Aktualisierung im Rebalancing-Tool (User-Direktive 09.06.:
"nur Updates der Beträge"). Teil der Umstrukturierung-2027-xlsx-Pflege.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Rebalancing_Tool_v3.4.xlsx
+++ b/03_Tools/Rebalancing_Tool_v3.4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tobia\OneDrive\Desktop\Claude Stuff\03_Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_ADF9235F583F999A114096030E7988BB87031414" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E117FD-7A60-4C74-829B-C782E3508459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1777,7 +1777,7 @@
     <row r="2" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="101">
         <f ca="1">TODAY()</f>
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B2" s="100"/>
       <c r="C2" s="100"/>
@@ -1869,11 +1869,11 @@
         <v>0</v>
       </c>
       <c r="F5" s="5">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="G5" s="6">
         <f t="shared" ref="G5:G23" si="0">IF(F$28=0,0,F5/F$28)</f>
-        <v>5.0827343424183699E-2</v>
+        <v>4.8214243907007237E-2</v>
       </c>
       <c r="H5" s="6">
         <f>'Parameter &amp; Regeln'!$B$56/'Parameter &amp; Regeln'!$B$4</f>
@@ -1881,15 +1881,15 @@
       </c>
       <c r="I5" s="5">
         <f t="shared" ref="I5:I23" si="1">H5*F$28</f>
-        <v>645.2494277400582</v>
+        <v>676.11654704170712</v>
       </c>
       <c r="J5" s="5">
         <f t="shared" ref="J5:J23" si="2">I5-F5</f>
-        <v>-17.750572259941805</v>
+        <v>17.116547041707122</v>
       </c>
       <c r="K5" s="6">
         <f t="shared" ref="K5:K23" si="3">G5-H5</f>
-        <v>1.360806081797665E-3</v>
+        <v>-1.2522934353787971E-3</v>
       </c>
       <c r="L5" s="3" t="str">
         <f>IF(C5="Aktie",IF(K5&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K5&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K5&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K5&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="G6" s="11">
         <f t="shared" si="0"/>
-        <v>0.30134098324460906</v>
+        <v>0.28758369817151685</v>
       </c>
       <c r="H6" s="11">
         <f>'Parameter &amp; Regeln'!$B$57/'Parameter &amp; Regeln'!$B$4</f>
@@ -1943,15 +1943,15 @@
       </c>
       <c r="I6" s="10">
         <f t="shared" si="1"/>
-        <v>3251.551037827352</v>
+        <v>3407.0971096023277</v>
       </c>
       <c r="J6" s="10">
         <f t="shared" si="2"/>
-        <v>-679.18896217264773</v>
+        <v>-523.64289039767209</v>
       </c>
       <c r="K6" s="11">
         <f t="shared" si="3"/>
-        <v>5.2068432323173569E-2</v>
+        <v>3.8311147250081362E-2</v>
       </c>
       <c r="L6" s="8" t="str">
         <f>IF(C6="Aktie",IF(K6&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K6&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K6&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K6&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="G7" s="11">
         <f t="shared" si="0"/>
-        <v>9.9080354733459275E-2</v>
+        <v>9.4556984992859319E-2</v>
       </c>
       <c r="H7" s="11">
         <f>'Parameter &amp; Regeln'!$B$58/'Parameter &amp; Regeln'!$B$4</f>
@@ -2005,15 +2005,15 @@
       </c>
       <c r="I7" s="10">
         <f t="shared" si="1"/>
-        <v>1556.1897963142578</v>
+        <v>1630.6340252182347</v>
       </c>
       <c r="J7" s="10">
         <f t="shared" si="2"/>
-        <v>263.76979631425775</v>
+        <v>338.21402521823461</v>
       </c>
       <c r="K7" s="11">
         <f t="shared" si="3"/>
-        <v>-2.0221294151118799E-2</v>
+        <v>-2.4744663891718754E-2</v>
       </c>
       <c r="L7" s="8" t="str">
         <f>IF(C7="Aktie",IF(K7&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K7&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K7&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K7&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="R7" s="94" t="str">
         <f>IF(AND(C7="Aktie",OR(LEFT(O7,1)="🔴",LEFT(N7,8)="DEFCON 1")),IF(J7&gt;'Parameter &amp; Regeln'!$B$64,"🚩 FLAG (gesperrt)",""),IF(J7&gt;'Parameter &amp; Regeln'!$B$64,"🛒 Nachkaufen",IF(J7&lt;-'Parameter &amp; Regeln'!$B$64,"⏸️ Über Ziel","")))</f>
-        <v/>
+        <v>🛒 Nachkaufen</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2055,11 +2055,11 @@
         <v>0.67</v>
       </c>
       <c r="F8" s="10">
-        <v>1323</v>
+        <v>1335</v>
       </c>
       <c r="G8" s="11">
         <f t="shared" si="0"/>
-        <v>0.10142469886907245</v>
+        <v>9.7672254348793106E-2</v>
       </c>
       <c r="H8" s="11">
         <f>'Parameter &amp; Regeln'!$B$59/'Parameter &amp; Regeln'!$B$4</f>
@@ -2067,15 +2067,15 @@
       </c>
       <c r="I8" s="10">
         <f t="shared" si="1"/>
-        <v>1303.1508050436471</v>
+        <v>1365.4902812803105</v>
       </c>
       <c r="J8" s="10">
         <f t="shared" si="2"/>
-        <v>-19.849194956352903</v>
+        <v>30.490281280310455</v>
       </c>
       <c r="K8" s="11">
         <f t="shared" si="3"/>
-        <v>1.5216920795477068E-3</v>
+        <v>-2.2307524407316343E-3</v>
       </c>
       <c r="L8" s="8" t="str">
         <f>IF(C8="Aktie",IF(K8&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K8&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K8&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K8&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2129,11 +2129,11 @@
       </c>
       <c r="I9" s="10">
         <f t="shared" si="1"/>
-        <v>1037.4598642095054</v>
+        <v>1087.0893501454898</v>
       </c>
       <c r="J9" s="10">
         <f t="shared" si="2"/>
-        <v>1037.4598642095054</v>
+        <v>1087.0893501454898</v>
       </c>
       <c r="K9" s="11">
         <f t="shared" si="3"/>
@@ -2179,11 +2179,11 @@
         <v>0.68</v>
       </c>
       <c r="F10" s="16">
-        <v>91</v>
+        <v>196</v>
       </c>
       <c r="G10" s="17">
         <f t="shared" si="0"/>
-        <v>6.9763020386134486E-3</v>
+        <v>1.4339896518624306E-2</v>
       </c>
       <c r="H10" s="17">
         <f>'Parameter &amp; Regeln'!$B$61/'Parameter &amp; Regeln'!$B$4</f>
@@ -2191,15 +2191,15 @@
       </c>
       <c r="I10" s="16">
         <f t="shared" si="1"/>
-        <v>645.2494277400582</v>
+        <v>676.11654704170712</v>
       </c>
       <c r="J10" s="16">
         <f t="shared" si="2"/>
-        <v>554.2494277400582</v>
+        <v>480.11654704170712</v>
       </c>
       <c r="K10" s="17">
         <f t="shared" si="3"/>
-        <v>-4.2490235303772585E-2</v>
+        <v>-3.5126640823761726E-2</v>
       </c>
       <c r="L10" s="14" t="str">
         <f>IF(C10="Aktie",IF(K10&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K10&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K10&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K10&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2241,11 +2241,11 @@
         <v>1</v>
       </c>
       <c r="F11" s="66">
-        <v>185</v>
+        <v>381</v>
       </c>
       <c r="G11" s="67">
         <f t="shared" si="0"/>
-        <v>1.4182592056521845E-2</v>
+        <v>2.7875002926509494E-2</v>
       </c>
       <c r="H11" s="67">
         <f>'Parameter &amp; Regeln'!$B$35/'Parameter &amp; Regeln'!$B$4</f>
@@ -2253,15 +2253,15 @@
       </c>
       <c r="I11" s="66">
         <f t="shared" si="1"/>
-        <v>506.07798254122213</v>
+        <v>530.28748787584868</v>
       </c>
       <c r="J11" s="66">
         <f t="shared" si="2"/>
-        <v>321.07798254122213</v>
+        <v>149.28748787584868</v>
       </c>
       <c r="K11" s="67">
         <f t="shared" si="3"/>
-        <v>-2.4614692133584852E-2</v>
+        <v>-1.0922281263597202E-2</v>
       </c>
       <c r="L11" s="64" t="str">
         <f>IF(C11="Aktie",IF(K11&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K11&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K11&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K11&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="R11" s="95" t="str">
         <f>IF(AND(C11="Aktie",OR(LEFT(O11,1)="🔴",LEFT(N11,8)="DEFCON 1")),IF(J11&gt;'Parameter &amp; Regeln'!$B$64,"🚩 FLAG (gesperrt)",""),IF(J11&gt;'Parameter &amp; Regeln'!$B$64,"🛒 Nachkaufen",IF(J11&lt;-'Parameter &amp; Regeln'!$B$64,"⏸️ Über Ziel","")))</f>
-        <v>🚩 FLAG (gesperrt)</v>
+        <v/>
       </c>
     </row>
     <row r="12" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2307,11 +2307,11 @@
         <v>1</v>
       </c>
       <c r="F12" s="68">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="G12" s="82">
         <f t="shared" si="0"/>
-        <v>2.5375340382209358E-2</v>
+        <v>2.5094818907592537E-2</v>
       </c>
       <c r="H12" s="82">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -2319,15 +2319,15 @@
       </c>
       <c r="I12" s="68">
         <f t="shared" si="1"/>
-        <v>227.73509214354996</v>
+        <v>238.62936954413192</v>
       </c>
       <c r="J12" s="68">
         <f t="shared" si="2"/>
-        <v>-103.26490785645004</v>
+        <v>-104.37063045586808</v>
       </c>
       <c r="K12" s="82">
         <f t="shared" si="3"/>
-        <v>7.916562496661346E-3</v>
+        <v>7.6360410220445256E-3</v>
       </c>
       <c r="L12" s="80" t="str">
         <f>IF(C12="Aktie",IF(K12&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K12&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K12&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K12&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2373,11 +2373,11 @@
         <v>0</v>
       </c>
       <c r="F13" s="66">
-        <v>486</v>
+        <v>519</v>
       </c>
       <c r="G13" s="67">
         <f t="shared" si="0"/>
-        <v>3.7258052645781713E-2</v>
+        <v>3.7971460679418444E-2</v>
       </c>
       <c r="H13" s="67">
         <f>'Parameter &amp; Regeln'!$B$36/'Parameter &amp; Regeln'!$B$4</f>
@@ -2385,15 +2385,15 @@
       </c>
       <c r="I13" s="66">
         <f t="shared" si="1"/>
-        <v>404.86238603297767</v>
+        <v>424.22999030067894</v>
       </c>
       <c r="J13" s="66">
         <f t="shared" si="2"/>
-        <v>-81.137613967022332</v>
+        <v>-94.770009699321065</v>
       </c>
       <c r="K13" s="67">
         <f t="shared" si="3"/>
-        <v>6.2202252936963583E-3</v>
+        <v>6.9336333273330893E-3</v>
       </c>
       <c r="L13" s="64" t="str">
         <f>IF(C13="Aktie",IF(K13&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K13&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K13&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K13&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2439,11 +2439,11 @@
         <v>1</v>
       </c>
       <c r="F14" s="68">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="G14" s="82">
         <f t="shared" si="0"/>
-        <v>3.4421534234477344E-2</v>
+        <v>3.2776906328284131E-2</v>
       </c>
       <c r="H14" s="82">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -2451,15 +2451,15 @@
       </c>
       <c r="I14" s="68">
         <f t="shared" si="1"/>
-        <v>227.73509214354996</v>
+        <v>238.62936954413192</v>
       </c>
       <c r="J14" s="68">
         <f t="shared" si="2"/>
-        <v>-221.26490785645004</v>
+        <v>-209.37063045586808</v>
       </c>
       <c r="K14" s="82">
         <f t="shared" si="3"/>
-        <v>1.6962756348929332E-2</v>
+        <v>1.5318128442736119E-2</v>
       </c>
       <c r="L14" s="80" t="str">
         <f>IF(C14="Aktie",IF(K14&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K14&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K14&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K14&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2505,11 +2505,11 @@
         <v>1</v>
       </c>
       <c r="F15" s="66">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="G15" s="67">
         <f t="shared" si="0"/>
-        <v>3.6261438068836936E-2</v>
+        <v>3.5557090347201087E-2</v>
       </c>
       <c r="H15" s="67">
         <f>'Parameter &amp; Regeln'!$B$35/'Parameter &amp; Regeln'!$B$4</f>
@@ -2517,15 +2517,15 @@
       </c>
       <c r="I15" s="66">
         <f t="shared" si="1"/>
-        <v>506.07798254122213</v>
+        <v>530.28748787584868</v>
       </c>
       <c r="J15" s="66">
         <f t="shared" si="2"/>
-        <v>33.077982541222127</v>
+        <v>44.287487875848683</v>
       </c>
       <c r="K15" s="67">
         <f t="shared" si="3"/>
-        <v>-2.5358461212697594E-3</v>
+        <v>-3.2401938429056087E-3</v>
       </c>
       <c r="L15" s="64" t="str">
         <f>IF(C15="Aktie",IF(K15&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K15&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K15&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K15&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2571,11 +2571,11 @@
         <v>0</v>
       </c>
       <c r="F16" s="68">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="G16" s="82">
         <f t="shared" si="0"/>
-        <v>3.0895051885288131E-2</v>
+        <v>2.9996722309367171E-2</v>
       </c>
       <c r="H16" s="82">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -2583,15 +2583,15 @@
       </c>
       <c r="I16" s="68">
         <f t="shared" si="1"/>
-        <v>227.73509214354996</v>
+        <v>238.62936954413192</v>
       </c>
       <c r="J16" s="68">
         <f t="shared" si="2"/>
-        <v>-175.26490785645004</v>
+        <v>-171.37063045586808</v>
       </c>
       <c r="K16" s="82">
         <f t="shared" si="3"/>
-        <v>1.3436273999740119E-2</v>
+        <v>1.2537944423819159E-2</v>
       </c>
       <c r="L16" s="80" t="str">
         <f>IF(C16="Aktie",IF(K16&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K16&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K16&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K16&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2649,11 +2649,11 @@
       </c>
       <c r="I17" s="66">
         <f t="shared" si="1"/>
-        <v>404.86238603297767</v>
+        <v>424.22999030067894</v>
       </c>
       <c r="J17" s="66">
         <f t="shared" si="2"/>
-        <v>404.86238603297767</v>
+        <v>424.22999030067894</v>
       </c>
       <c r="K17" s="67">
         <f t="shared" si="3"/>
@@ -2703,11 +2703,11 @@
         <v>1</v>
       </c>
       <c r="F18" s="68">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="G18" s="82">
         <f t="shared" si="0"/>
-        <v>3.2964943698942671E-2</v>
+        <v>3.1094163369465969E-2</v>
       </c>
       <c r="H18" s="82">
         <f>'Parameter &amp; Regeln'!$B$35/'Parameter &amp; Regeln'!$B$4</f>
@@ -2715,15 +2715,15 @@
       </c>
       <c r="I18" s="68">
         <f t="shared" si="1"/>
-        <v>506.07798254122213</v>
+        <v>530.28748787584868</v>
       </c>
       <c r="J18" s="68">
         <f t="shared" si="2"/>
-        <v>76.077982541222127</v>
+        <v>105.28748787584868</v>
       </c>
       <c r="K18" s="82">
         <f t="shared" si="3"/>
-        <v>-5.8323404911640245E-3</v>
+        <v>-7.7031208206407263E-3</v>
       </c>
       <c r="L18" s="80" t="str">
         <f>IF(C18="Aktie",IF(K18&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K18&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K18&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K18&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2769,11 +2769,11 @@
         <v>0</v>
       </c>
       <c r="F19" s="66">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="G19" s="67">
         <f t="shared" si="0"/>
-        <v>3.1508353163407991E-2</v>
+        <v>3.058202420808653E-2</v>
       </c>
       <c r="H19" s="67">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -2781,15 +2781,15 @@
       </c>
       <c r="I19" s="66">
         <f t="shared" si="1"/>
-        <v>227.73509214354996</v>
+        <v>238.62936954413192</v>
       </c>
       <c r="J19" s="66">
         <f t="shared" si="2"/>
-        <v>-183.26490785645004</v>
+        <v>-179.37063045586808</v>
       </c>
       <c r="K19" s="67">
         <f t="shared" si="3"/>
-        <v>1.404957527785998E-2</v>
+        <v>1.3123246322538518E-2</v>
       </c>
       <c r="L19" s="64" t="str">
         <f>IF(C19="Aktie",IF(K19&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K19&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K19&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K19&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2835,11 +2835,11 @@
         <v>1</v>
       </c>
       <c r="F20" s="68">
-        <v>194</v>
+        <v>451</v>
       </c>
       <c r="G20" s="82">
         <f t="shared" si="0"/>
-        <v>1.4872555994406693E-2</v>
+        <v>3.299639454030389E-2</v>
       </c>
       <c r="H20" s="82">
         <f>'Parameter &amp; Regeln'!$B$35/'Parameter &amp; Regeln'!$B$4</f>
@@ -2847,15 +2847,15 @@
       </c>
       <c r="I20" s="68">
         <f t="shared" si="1"/>
-        <v>506.07798254122213</v>
+        <v>530.28748787584868</v>
       </c>
       <c r="J20" s="68">
         <f t="shared" si="2"/>
-        <v>312.07798254122213</v>
+        <v>79.287487875848683</v>
       </c>
       <c r="K20" s="82">
         <f t="shared" si="3"/>
-        <v>-2.3924728195700004E-2</v>
+        <v>-5.8008896498028054E-3</v>
       </c>
       <c r="L20" s="80" t="str">
         <f>IF(C20="Aktie",IF(K20&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K20&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K20&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K20&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="R20" s="96" t="str">
         <f>IF(AND(C20="Aktie",OR(LEFT(O20,1)="🔴",LEFT(N20,8)="DEFCON 1")),IF(J20&gt;'Parameter &amp; Regeln'!$B$64,"🚩 FLAG (gesperrt)",""),IF(J20&gt;'Parameter &amp; Regeln'!$B$64,"🛒 Nachkaufen",IF(J20&lt;-'Parameter &amp; Regeln'!$B$64,"⏸️ Über Ziel","")))</f>
-        <v>🛒 Nachkaufen</v>
+        <v/>
       </c>
     </row>
     <row r="21" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2901,11 +2901,11 @@
         <v>1</v>
       </c>
       <c r="F21" s="66">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="G21" s="67">
         <f t="shared" si="0"/>
-        <v>3.0665063905993179E-2</v>
+        <v>2.8972443986608292E-2</v>
       </c>
       <c r="H21" s="67">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -2913,15 +2913,15 @@
       </c>
       <c r="I21" s="66">
         <f t="shared" si="1"/>
-        <v>227.73509214354996</v>
+        <v>238.62936954413192</v>
       </c>
       <c r="J21" s="66">
         <f t="shared" si="2"/>
-        <v>-172.26490785645004</v>
+        <v>-157.37063045586808</v>
       </c>
       <c r="K21" s="67">
         <f t="shared" si="3"/>
-        <v>1.3206286020445168E-2</v>
+        <v>1.151366610106028E-2</v>
       </c>
       <c r="L21" s="64" t="str">
         <f>IF(C21="Aktie",IF(K21&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K21&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K21&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K21&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2967,11 +2967,11 @@
         <v>1</v>
       </c>
       <c r="F22" s="68">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="G22" s="82">
         <f t="shared" si="0"/>
-        <v>3.6798076687191816E-2</v>
+        <v>3.4752300236461968E-2</v>
       </c>
       <c r="H22" s="82">
         <f>'Parameter &amp; Regeln'!$B$36/'Parameter &amp; Regeln'!$B$4</f>
@@ -2979,15 +2979,15 @@
       </c>
       <c r="I22" s="68">
         <f t="shared" si="1"/>
-        <v>404.86238603297767</v>
+        <v>424.22999030067894</v>
       </c>
       <c r="J22" s="68">
         <f t="shared" si="2"/>
-        <v>-75.137613967022332</v>
+        <v>-50.770009699321065</v>
       </c>
       <c r="K22" s="82">
         <f t="shared" si="3"/>
-        <v>5.7602493351064619E-3</v>
+        <v>3.7144728843766135E-3</v>
       </c>
       <c r="L22" s="80" t="str">
         <f>IF(C22="Aktie",IF(K22&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K22&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K22&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K22&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3033,11 +3033,11 @@
         <v>1</v>
       </c>
       <c r="F23" s="66">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G23" s="67">
         <f t="shared" si="0"/>
-        <v>3.6108112749306968E-2</v>
+        <v>3.4532812024442208E-2</v>
       </c>
       <c r="H23" s="67">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -3045,15 +3045,15 @@
       </c>
       <c r="I23" s="66">
         <f t="shared" si="1"/>
-        <v>227.73509214354996</v>
+        <v>238.62936954413192</v>
       </c>
       <c r="J23" s="66">
         <f t="shared" si="2"/>
-        <v>-243.26490785645004</v>
+        <v>-233.37063045586808</v>
       </c>
       <c r="K23" s="67">
         <f t="shared" si="3"/>
-        <v>1.8649334863758957E-2</v>
+        <v>1.7074034138894197E-2</v>
       </c>
       <c r="L23" s="64" t="str">
         <f>IF(C23="Aktie",IF(K23&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K23&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K23&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K23&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3092,11 +3092,11 @@
       <c r="E24" s="19"/>
       <c r="F24" s="20">
         <f>SUM(F5:F23)</f>
-        <v>12013.16</v>
+        <v>12637.16</v>
       </c>
       <c r="G24" s="21">
         <f>SUM(G5:G23)</f>
-        <v>0.92096079778230266</v>
+        <v>0.92456921780254253</v>
       </c>
       <c r="H24" s="21">
         <f>SUM(H5:H23)</f>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="I24" s="20">
         <f>SUM(I5:I23)</f>
-        <v>13044.160000000002</v>
+        <v>13668.160000000003</v>
       </c>
       <c r="J24" s="20">
         <f>ROUND(SUM(J5:J23),2)</f>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="K24" s="21">
         <f t="array" ref="K24">SUMPRODUCT((C5:C23="Aktie")*ABS(K5:K23))/COUNTIF(C5:C23,"Aktie")</f>
-        <v>1.4165130610000132E-2</v>
+        <v>1.1273498430141091E-2</v>
       </c>
       <c r="L24" s="18" t="s">
         <v>83</v>
@@ -3137,7 +3137,7 @@
     <row r="25" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K25" s="24">
         <f t="array" ref="K25">SUMPRODUCT((C5:C23&lt;&gt;"Aktie")*ABS(K5:K23))/COUNTIF(C5:C23,"&lt;&gt;Aktie")</f>
-        <v>3.2866148754854836E-2</v>
+        <v>3.0199988405231831E-2</v>
       </c>
       <c r="L25" s="25" t="s">
         <v>84</v>
@@ -3178,7 +3178,7 @@
       </c>
       <c r="F28" s="33">
         <f>F24 + F27</f>
-        <v>13044.16</v>
+        <v>13668.16</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="C4" s="39">
         <f>'Portfolio &amp; Rebalancing'!F5</f>
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="D4" s="40">
         <f>'Portfolio &amp; Rebalancing'!E5</f>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="C7" s="39">
         <f>'Portfolio &amp; Rebalancing'!F8</f>
-        <v>1323</v>
+        <v>1335</v>
       </c>
       <c r="D7" s="40">
         <f>'Portfolio &amp; Rebalancing'!E8</f>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="E7" s="39">
         <f t="shared" si="0"/>
-        <v>886.41000000000008</v>
+        <v>894.45</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="C9" s="39">
         <f>'Portfolio &amp; Rebalancing'!F10</f>
-        <v>91</v>
+        <v>196</v>
       </c>
       <c r="D9" s="40">
         <f>'Portfolio &amp; Rebalancing'!E10</f>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="E9" s="39">
         <f t="shared" si="0"/>
-        <v>61.88</v>
+        <v>133.28</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="C10" s="39">
         <f>'Portfolio &amp; Rebalancing'!F11</f>
-        <v>185</v>
+        <v>381</v>
       </c>
       <c r="D10" s="40">
         <f>'Portfolio &amp; Rebalancing'!E11</f>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="E10" s="39">
         <f t="shared" si="0"/>
-        <v>185</v>
+        <v>381</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="C11" s="39">
         <f>'Portfolio &amp; Rebalancing'!F12</f>
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="D11" s="40">
         <f>'Portfolio &amp; Rebalancing'!E12</f>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="E11" s="39">
         <f t="shared" si="0"/>
-        <v>331</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="C12" s="39">
         <f>'Portfolio &amp; Rebalancing'!F13</f>
-        <v>486</v>
+        <v>519</v>
       </c>
       <c r="D12" s="40">
         <f>'Portfolio &amp; Rebalancing'!E13</f>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="C13" s="39">
         <f>'Portfolio &amp; Rebalancing'!F14</f>
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D13" s="40">
         <f>'Portfolio &amp; Rebalancing'!E14</f>
@@ -3549,7 +3549,7 @@
       </c>
       <c r="E13" s="39">
         <f t="shared" si="0"/>
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="C14" s="39">
         <f>'Portfolio &amp; Rebalancing'!F15</f>
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="D14" s="40">
         <f>'Portfolio &amp; Rebalancing'!E15</f>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="E14" s="39">
         <f t="shared" si="0"/>
-        <v>473</v>
+        <v>486</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="C15" s="39">
         <f>'Portfolio &amp; Rebalancing'!F16</f>
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="D15" s="40">
         <f>'Portfolio &amp; Rebalancing'!E16</f>
@@ -3629,7 +3629,7 @@
       </c>
       <c r="C17" s="39">
         <f>'Portfolio &amp; Rebalancing'!F18</f>
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="D17" s="40">
         <f>'Portfolio &amp; Rebalancing'!E18</f>
@@ -3637,7 +3637,7 @@
       </c>
       <c r="E17" s="39">
         <f t="shared" si="0"/>
-        <v>430</v>
+        <v>425</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="C18" s="39">
         <f>'Portfolio &amp; Rebalancing'!F19</f>
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="D18" s="40">
         <f>'Portfolio &amp; Rebalancing'!E19</f>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="C19" s="39">
         <f>'Portfolio &amp; Rebalancing'!F20</f>
-        <v>194</v>
+        <v>451</v>
       </c>
       <c r="D19" s="40">
         <f>'Portfolio &amp; Rebalancing'!E20</f>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="E19" s="39">
         <f t="shared" si="0"/>
-        <v>194</v>
+        <v>451</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="C20" s="39">
         <f>'Portfolio &amp; Rebalancing'!F21</f>
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="D20" s="40">
         <f>'Portfolio &amp; Rebalancing'!E21</f>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="E20" s="39">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="C21" s="39">
         <f>'Portfolio &amp; Rebalancing'!F22</f>
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="D21" s="40">
         <f>'Portfolio &amp; Rebalancing'!E22</f>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="E21" s="39">
         <f t="shared" si="0"/>
-        <v>480</v>
+        <v>475</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -3739,7 +3739,7 @@
       </c>
       <c r="C22" s="39">
         <f>'Portfolio &amp; Rebalancing'!F23</f>
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D22" s="40">
         <f>'Portfolio &amp; Rebalancing'!E23</f>
@@ -3747,7 +3747,7 @@
       </c>
       <c r="E22" s="39">
         <f t="shared" si="0"/>
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -3757,11 +3757,11 @@
       </c>
       <c r="C23" s="42">
         <f>'Portfolio &amp; Rebalancing'!F24</f>
-        <v>12013.16</v>
+        <v>12637.16</v>
       </c>
       <c r="E23" s="42">
         <f>SUM(E4:E22)</f>
-        <v>7112.808</v>
+        <v>7656.2479999999996</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="B25" s="43">
         <f>IF('Portfolio &amp; Rebalancing'!F24=0,0,E23/'Portfolio &amp; Rebalancing'!F24)</f>
-        <v>0.59208468046708773</v>
+        <v>0.60585194774775342</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="B26" s="43">
         <f>SUMPRODUCT('Portfolio &amp; Rebalancing'!$E$5:$E$23,'Portfolio &amp; Rebalancing'!$I$5:$I$23)/SUM('Portfolio &amp; Rebalancing'!$I$5:$I$23)</f>
-        <v>0.58043646944713867</v>
+        <v>0.58043646944713845</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>